<commit_message>
fix(e2e): rebuild Excel fixture with correct header rows per sheet
</commit_message>
<xml_diff>
--- a/backend/e2e/fixtures/test_data.xlsx
+++ b/backend/e2e/fixtures/test_data.xlsx
@@ -417,419 +417,418 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BQ3"/>
+  <dimension ref="A2:BP3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="B1" t="inlineStr">
+    <row r="2">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Week</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Team</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>COORD.</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Date2</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Po</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Style</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Batch</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Color</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Column2</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>Seconds</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>Rejected</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>Sample</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>Defects</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>AQL %</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>Pass/Fail</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>Def19</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>Def20</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>Def21</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>Def22</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>Def23</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>Def24</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>Def25</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>Def26</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>Def27</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>Def28</t>
-        </is>
-      </c>
-      <c r="AE1" t="inlineStr">
-        <is>
-          <t>Def29</t>
-        </is>
-      </c>
-      <c r="AF1" t="inlineStr">
-        <is>
-          <t>Def30</t>
-        </is>
-      </c>
-      <c r="AG1" t="inlineStr">
-        <is>
-          <t>Def31</t>
-        </is>
-      </c>
-      <c r="AH1" t="inlineStr">
-        <is>
-          <t>Def32</t>
-        </is>
-      </c>
-      <c r="AI1" t="inlineStr">
-        <is>
-          <t>Def33</t>
-        </is>
-      </c>
-      <c r="AJ1" t="inlineStr">
-        <is>
-          <t>Def34</t>
-        </is>
-      </c>
-      <c r="AK1" t="inlineStr">
-        <is>
-          <t>Def35</t>
-        </is>
-      </c>
-      <c r="AL1" t="inlineStr">
-        <is>
-          <t>Def36</t>
-        </is>
-      </c>
-      <c r="AM1" t="inlineStr">
-        <is>
-          <t>Def37</t>
-        </is>
-      </c>
-      <c r="AN1" t="inlineStr">
-        <is>
-          <t>Def38</t>
-        </is>
-      </c>
-      <c r="AO1" t="inlineStr">
-        <is>
-          <t>Def39</t>
-        </is>
-      </c>
-      <c r="AP1" t="inlineStr">
-        <is>
-          <t>Def40</t>
-        </is>
-      </c>
-      <c r="AQ1" t="inlineStr">
-        <is>
-          <t>Def41</t>
-        </is>
-      </c>
-      <c r="AR1" t="inlineStr">
-        <is>
-          <t>Def42</t>
-        </is>
-      </c>
-      <c r="AS1" t="inlineStr">
-        <is>
-          <t>Def43</t>
-        </is>
-      </c>
-      <c r="AT1" t="inlineStr">
-        <is>
-          <t>Def44</t>
-        </is>
-      </c>
-      <c r="AU1" t="inlineStr">
-        <is>
-          <t>Def45</t>
-        </is>
-      </c>
-      <c r="AV1" t="inlineStr">
-        <is>
-          <t>Def46</t>
-        </is>
-      </c>
-      <c r="AW1" t="inlineStr">
-        <is>
-          <t>Def47</t>
-        </is>
-      </c>
-      <c r="AX1" t="inlineStr">
-        <is>
-          <t>Def48</t>
-        </is>
-      </c>
-      <c r="AY1" t="inlineStr">
-        <is>
-          <t>Def49</t>
-        </is>
-      </c>
-      <c r="AZ1" t="inlineStr">
-        <is>
-          <t>Def50</t>
-        </is>
-      </c>
-      <c r="BA1" t="inlineStr">
-        <is>
-          <t>Def51</t>
-        </is>
-      </c>
-      <c r="BB1" t="inlineStr">
-        <is>
-          <t>Def52</t>
-        </is>
-      </c>
-      <c r="BC1" t="inlineStr">
-        <is>
-          <t>Def53</t>
-        </is>
-      </c>
-      <c r="BD1" t="inlineStr">
-        <is>
-          <t>Def54</t>
-        </is>
-      </c>
-      <c r="BE1" t="inlineStr">
-        <is>
-          <t>Def55</t>
-        </is>
-      </c>
-      <c r="BF1" t="inlineStr">
-        <is>
-          <t>Def56</t>
-        </is>
-      </c>
-      <c r="BG1" t="inlineStr">
-        <is>
-          <t>Def57</t>
-        </is>
-      </c>
-      <c r="BH1" t="inlineStr">
-        <is>
-          <t>Def58</t>
-        </is>
-      </c>
-      <c r="BI1" t="inlineStr">
-        <is>
-          <t>Def59</t>
-        </is>
-      </c>
-      <c r="BJ1" t="inlineStr">
-        <is>
-          <t>Def60</t>
-        </is>
-      </c>
-      <c r="BK1" t="inlineStr">
-        <is>
-          <t>Def61</t>
-        </is>
-      </c>
-      <c r="BL1" t="inlineStr">
-        <is>
-          <t>Def62</t>
-        </is>
-      </c>
-      <c r="BM1" t="inlineStr">
-        <is>
-          <t>Def63</t>
-        </is>
-      </c>
-      <c r="BN1" t="inlineStr">
-        <is>
-          <t>Def64</t>
-        </is>
-      </c>
-      <c r="BO1" t="inlineStr">
-        <is>
-          <t>Def65</t>
-        </is>
-      </c>
-      <c r="BP1" t="inlineStr">
-        <is>
-          <t>Def66</t>
-        </is>
-      </c>
-      <c r="BQ1" t="inlineStr">
-        <is>
-          <t>Def67</t>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>D19</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>D20</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>D21</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>D22</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>D23</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>D24</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>D25</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>D26</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>D27</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>D28</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>D29</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>D30</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>D31</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>D32</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>D33</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>D34</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>D35</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>D36</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>D37</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>D38</t>
+        </is>
+      </c>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>D39</t>
+        </is>
+      </c>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>D40</t>
+        </is>
+      </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>D41</t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t>D42</t>
+        </is>
+      </c>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t>D43</t>
+        </is>
+      </c>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>D44</t>
+        </is>
+      </c>
+      <c r="AT2" t="inlineStr">
+        <is>
+          <t>D45</t>
+        </is>
+      </c>
+      <c r="AU2" t="inlineStr">
+        <is>
+          <t>D46</t>
+        </is>
+      </c>
+      <c r="AV2" t="inlineStr">
+        <is>
+          <t>D47</t>
+        </is>
+      </c>
+      <c r="AW2" t="inlineStr">
+        <is>
+          <t>D48</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>D49</t>
+        </is>
+      </c>
+      <c r="AY2" t="inlineStr">
+        <is>
+          <t>D50</t>
+        </is>
+      </c>
+      <c r="AZ2" t="inlineStr">
+        <is>
+          <t>D51</t>
+        </is>
+      </c>
+      <c r="BA2" t="inlineStr">
+        <is>
+          <t>D52</t>
+        </is>
+      </c>
+      <c r="BB2" t="inlineStr">
+        <is>
+          <t>D53</t>
+        </is>
+      </c>
+      <c r="BC2" t="inlineStr">
+        <is>
+          <t>D54</t>
+        </is>
+      </c>
+      <c r="BD2" t="inlineStr">
+        <is>
+          <t>D55</t>
+        </is>
+      </c>
+      <c r="BE2" t="inlineStr">
+        <is>
+          <t>D56</t>
+        </is>
+      </c>
+      <c r="BF2" t="inlineStr">
+        <is>
+          <t>D57</t>
+        </is>
+      </c>
+      <c r="BG2" t="inlineStr">
+        <is>
+          <t>D58</t>
+        </is>
+      </c>
+      <c r="BH2" t="inlineStr">
+        <is>
+          <t>D59</t>
+        </is>
+      </c>
+      <c r="BI2" t="inlineStr">
+        <is>
+          <t>D60</t>
+        </is>
+      </c>
+      <c r="BJ2" t="inlineStr">
+        <is>
+          <t>D61</t>
+        </is>
+      </c>
+      <c r="BK2" t="inlineStr">
+        <is>
+          <t>D62</t>
+        </is>
+      </c>
+      <c r="BL2" t="inlineStr">
+        <is>
+          <t>D63</t>
+        </is>
+      </c>
+      <c r="BM2" t="inlineStr">
+        <is>
+          <t>D64</t>
+        </is>
+      </c>
+      <c r="BN2" t="inlineStr">
+        <is>
+          <t>D65</t>
+        </is>
+      </c>
+      <c r="BO2" t="inlineStr">
+        <is>
+          <t>D66</t>
+        </is>
+      </c>
+      <c r="BP2" t="inlineStr">
+        <is>
+          <t>D67</t>
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>2025-01-15</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="B3" t="n">
         <v>3</v>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>CUST</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="D3" t="n">
         <v>1</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="n">
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="n">
         <v>123</v>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>STYLE1</t>
         </is>
       </c>
-      <c r="J3" t="n">
+      <c r="I3" t="n">
         <v>1</v>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>RED</t>
         </is>
       </c>
-      <c r="L3" t="n">
+      <c r="K3" t="n">
         <v>100</v>
       </c>
-      <c r="M3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
       <c r="N3" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="O3" t="n">
-        <v>80</v>
+        <v>20</v>
       </c>
       <c r="P3" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="Q3" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="R3" t="n">
-        <v>10</v>
-      </c>
-      <c r="S3" t="n">
         <v>1.5</v>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
+      <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr"/>
@@ -877,7 +876,6 @@
       <c r="BM3" t="inlineStr"/>
       <c r="BN3" t="inlineStr"/>
       <c r="BO3" t="inlineStr"/>
-      <c r="BP3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1226,195 +1224,194 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W2"/>
+  <dimension ref="A2:V3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="B1" t="inlineStr">
+    <row r="2">
+      <c r="A2" t="inlineStr">
         <is>
           <t>year</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>week</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>DATE</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>CUT#</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>STYLE</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>CUT QTY</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>COLOR</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>FIRST QUALITY QTY SEWING</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Sample</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>SEW DEF.</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>FAB. DEF.</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>% ACEPTED</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>% REJECTED</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>TOTAL OF 2DS</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>% OF 2DS</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>LINE#</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>2DA BY SEW</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>2DA BY  FAB</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>%Seconds Sew A4</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="V2" t="inlineStr">
         <is>
           <t>%Seconds Fab A4</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="n">
+    <row r="3">
+      <c r="A3" t="n">
         <v>2025</v>
       </c>
-      <c r="C2" t="n">
+      <c r="B3" t="n">
         <v>3</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>2025-01-15</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="D3" t="n">
         <v>1</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>STYLE1</t>
         </is>
       </c>
-      <c r="G2" t="n">
+      <c r="F3" t="n">
         <v>500</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>RED</t>
         </is>
       </c>
-      <c r="I2" t="n">
+      <c r="H3" t="n">
         <v>400</v>
       </c>
-      <c r="J2" t="n">
+      <c r="I3" t="n">
         <v>50</v>
       </c>
-      <c r="K2" t="n">
+      <c r="J3" t="n">
         <v>45</v>
       </c>
-      <c r="L2" t="n">
+      <c r="K3" t="n">
         <v>5</v>
       </c>
-      <c r="M2" t="n">
+      <c r="L3" t="n">
         <v>10</v>
       </c>
-      <c r="N2" t="n">
+      <c r="M3" t="n">
         <v>5</v>
       </c>
-      <c r="O2" t="n">
+      <c r="N3" t="n">
         <v>90</v>
       </c>
-      <c r="P2" t="n">
+      <c r="O3" t="n">
         <v>10</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="P3" t="n">
         <v>15</v>
       </c>
-      <c r="R2" t="n">
+      <c r="Q3" t="n">
         <v>5</v>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>L1</t>
         </is>
       </c>
-      <c r="T2" t="n">
+      <c r="S3" t="n">
         <v>100</v>
       </c>
-      <c r="U2" t="n">
+      <c r="T3" t="n">
         <v>50</v>
       </c>
-      <c r="V2" t="n">
+      <c r="U3" t="n">
         <v>10</v>
       </c>
-      <c r="W2" t="n">
+      <c r="V3" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1429,276 +1426,275 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM2"/>
+  <dimension ref="A2:AL3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="B1" t="inlineStr">
+    <row r="2">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Week</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Line</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Style</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>ArtCode</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Color</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t xml:space="preserve">PO </t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Size</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Produced</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Definitive</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>D13</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>D14</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>D15</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>D16</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>D17</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>D18</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>D19</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>D20</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>D21</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>D22</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>D23</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>D24</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>D25</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>D26</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>D27</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>D28</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>D29</t>
-        </is>
-      </c>
-      <c r="AE1" t="inlineStr">
-        <is>
-          <t>D30</t>
-        </is>
-      </c>
-      <c r="AF1" t="inlineStr">
-        <is>
-          <t>D31</t>
-        </is>
-      </c>
-      <c r="AG1" t="inlineStr">
-        <is>
-          <t>D32</t>
-        </is>
-      </c>
-      <c r="AH1" t="inlineStr">
-        <is>
-          <t>D33</t>
-        </is>
-      </c>
-      <c r="AI1" t="inlineStr">
-        <is>
-          <t>D34</t>
-        </is>
-      </c>
-      <c r="AJ1" t="inlineStr">
-        <is>
-          <t>D35</t>
-        </is>
-      </c>
-      <c r="AK1" t="inlineStr">
-        <is>
-          <t>D36</t>
-        </is>
-      </c>
-      <c r="AL1" t="inlineStr">
-        <is>
-          <t>D37</t>
-        </is>
-      </c>
-      <c r="AM1" t="inlineStr">
-        <is>
-          <t>D38</t>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Picado de Aguja</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Manchas/Sucio</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Grasa</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Tono Tela</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Fuera Medidas</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Enganche</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Costura Torcida/Insegura</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Hoyos Costura</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Heat Transfer Defectuoso/Inclinado/Fuera de Posicion</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Mal Corte</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Trapo</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>Corrido</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>Otros</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>Total De Costura</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>Desgarre/Def Tela</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>Contamination</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>Linea de Tela</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>Mill  Flaw</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>Hoyos</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>Manchas Tela</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>Corrido2</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>Barre</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>Otros3</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>Degradacion</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>Bordados</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>Total de Tela</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr">
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
           <t>2025-01-15</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="B3" t="n">
         <v>3</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>L1</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>CUST</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>STYLE1</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
         <is>
           <t>RED</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>123</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="K2" t="n">
+      <c r="J3" t="n">
         <v>100</v>
       </c>
-      <c r="L2" t="n">
+      <c r="K3" t="n">
         <v>0</v>
       </c>
-      <c r="M2" t="n">
+      <c r="L3" t="n">
         <v>100</v>
       </c>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr"/>
-      <c r="AL2" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr"/>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
+      <c r="AG3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr"/>
+      <c r="AJ3" t="inlineStr"/>
+      <c r="AK3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1711,179 +1707,177 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z2"/>
+  <dimension ref="A3:X4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="C1" t="inlineStr">
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t># Container</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t># Transfert of Container</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Total Palette</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Total Palette Pass</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Total Palette reject</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>% Pass</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>% Reject</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>C10</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>C11</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>C12</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>C13</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>C14</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>C15</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>C16</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>C17</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>C18</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>C19</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>C20</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>C21</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>C22</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>C23</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>C24</t>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Dirt label/ Salte nan Etikèt</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>dirt container/ Konntenè sal</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Dirt Cartons/ Katon Sal</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Container Holes Twou nan Konntenè</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Written mark on Label Ekriti sou Etikèt</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Written mark on Carton Ekriti sou Bwat yo</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>container poor close Kontenè mal fèmen</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>boxes pooor close Bwat ki mal fèmen</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Printing Issues label/ Problem Enpresyon Etikèt</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Misaligned label/ Etikèt kwochi</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Crushed corners Boxes / Bwat kraze</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Cartons Holes Twou nan Bwat2</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>Warped Boxes/ Bwat Defòme</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>Defects label carton /Defo Etikèt katon</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>Total defects</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>2025-01-15</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="B4" t="n">
         <v>1001</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>CUST</t>
         </is>
       </c>
-      <c r="F2" t="n">
+      <c r="D4" t="n">
         <v>5</v>
       </c>
-      <c r="G2" t="n">
+      <c r="E4" t="n">
         <v>10</v>
       </c>
-      <c r="H2" t="n">
+      <c r="F4" t="n">
         <v>8</v>
       </c>
-      <c r="I2" t="n">
+      <c r="G4" t="n">
         <v>2</v>
       </c>
-      <c r="J2" t="n">
+      <c r="H4" t="n">
         <v>80</v>
       </c>
-      <c r="K2" t="n">
+      <c r="I4" t="n">
         <v>20</v>
       </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>